<commit_message>
2 157 chaines, 306 630 videos, 257 preuves fortes
La moisson a ete arretee trois fois par l environnement, jamais par une erreur
de code : la reprise reparee ce matin a chaque fois tout retrouve. Elle est a
2 157 chaines sur 2 660.

A_VERIFIER_3.xlsx passe de 72 a 82 candidats jamais vus. ETAT.md porte
desormais le point de reprise exact, pour qu une session suivante n ait pas a
le deviner.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DfPtphAAkK24cZ5SByH1EW
</commit_message>
<xml_diff>
--- a/cartographie/A_VERIFIER_3.xlsx
+++ b/cartographie/A_VERIFIER_3.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="a verifier" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'a verifier'!$A$1:$K$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'a verifier'!$A$1:$K$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4090,10 +4090,490 @@
       <c r="J73" s="8" t="inlineStr"/>
       <c r="K73" s="8" t="inlineStr"/>
     </row>
+    <row r="74" ht="108" customHeight="1">
+      <c r="A74" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Coopérative U</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="n">
+        <v>11800</v>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>PRODUITS U | Origine France | Lait Français | Pas de jalouse</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>Yaourts, beurre, crème, fromage ou lait frais...chez Coopérative U, les produits laitiers U du rayon frais sont au lait Français*. 
+Comme par exemple cet emmental râpé U.
+*Hors spécialités étrangères et fromages fondus.
+🔔 Abonnez-vous à notre chaîne YouTube pour plus de vidéos :
+http://https://www.youtube.com/@CooperativeU/
+Pour plus de contenus, retrouvez-nous aussi par ici :
+TikTok : https://www.tiktok.com/coo</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J74" s="8" t="inlineStr"/>
+      <c r="K74" s="8" t="inlineStr"/>
+    </row>
+    <row r="75" ht="108" customHeight="1">
+      <c r="A75" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Coopérative U</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="n">
+        <v>11800</v>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>PRODUITS U | Origine France | Lait Français | Les filles</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>Yaourts, beurre, crème, fromage ou lait frais...chez Coopérative U, les produits laitiers U du rayon frais sont au lait Français*. 
+Comme par exemple ces yaourts nature U.
+*Hors spécialités étrangères et fromages fondus.
+🔔 Abonnez-vous à notre chaîne YouTube pour plus de vidéos :
+http://https://www.youtube.com/@CooperativeU/
+Pour plus de contenus, retrouvez-nous aussi par ici :
+TikTok : https://www.tiktok.com/co</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J75" s="8" t="inlineStr"/>
+      <c r="K75" s="8" t="inlineStr"/>
+    </row>
+    <row r="76" ht="108" customHeight="1">
+      <c r="A76" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Claire Sauzel</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="n">
+        <v>9860</v>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>2021-06-10</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>une journée dans mon assiette! 🦋 RECETTES HEALTHY et FACILES (Acai Bowl, Ramen, Tacos, Iced Latte)</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>...à l'autre et je suis aucun régime je mange intuitivement, j'évite simplement le gluten et les produits laitiers pour des questions de digestion et de ballonnement. Ici je vous montre comment faire un porridge (oatmeal),  la recette de tacos salade ou taco lettuce wraps, mon iced latte, un assai bowl style nice cream, et ma recette de ramen végétarien! Des recettes saines, healthy, et nourrissantes! 
+OATMEAL (porridge) : https://www.ins</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J76" s="8" t="inlineStr"/>
+      <c r="K76" s="8" t="inlineStr"/>
+    </row>
+    <row r="77" ht="108" customHeight="1">
+      <c r="A77" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Claire Sauzel</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="n">
+        <v>9860</v>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>2021-06-04</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>une journée dans mon assiette + RECETTES D'ETE HEALTHY ET FACILES (Twix Healthy, Green Smoothie)</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>...à l'autre et je suis aucun régime je mange intuitivement, j'évite simplement le gluten et les produits laitiers pour des questions de digestion et de ballonnement. Ici je vous montre comment faire un smoothie green crémeux et épais avec des épinards et des bananes congelées, mais aussi comment faire des galettes de thon healthy et ma salade préférée pour l'été, la salade pastèque et feta avec du lime! Enfin je partage ma recette de Twix</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J77" s="8" t="inlineStr"/>
+      <c r="K77" s="8" t="inlineStr"/>
+    </row>
+    <row r="78" ht="108" customHeight="1">
+      <c r="A78" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Margaux Lifestyle | Running, SOPK &amp; Lipœdème</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="n">
+        <v>4570</v>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>2025-10-26</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Mon petit déjeuner SOPK friendly : un chia porridge avec du GYN OPK</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>...3 c. à s. de graines de chia
+- 1 sachet de GYN OPK
+- 200 ml de lait (végétal si tu évites les produits laitiers)
+→ Mélanger, laisser gonfler 5–10 min, remélanger pour homogénéiser
+- 100 g de framboises surgelées
+→ Laisser reposer toute la nuit au frigo
+🌞 Le matin : ajouter 15 amandes + 1 carré de chocolat noir 🍫
+💡 Bienfaits :
+👉 Graines de chia → fibres, oméga-3 et satiété
+👉 GYN OPK → soutien hormonal et métabolique
+👉 Framboises → faibl</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="J78" s="8" t="inlineStr"/>
+      <c r="K78" s="8" t="inlineStr"/>
+    </row>
+    <row r="79" ht="108" customHeight="1">
+      <c r="A79" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>My Boucherie</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>2024-06-13</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>Rumsteck persillé 😍 #legrascestlavie #jaimelaviande #frenchbutcher #marseilleboucheriecapel</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J79" s="8" t="inlineStr"/>
+      <c r="K79" s="8" t="inlineStr"/>
+    </row>
+    <row r="80" ht="108" customHeight="1">
+      <c r="A80" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Toscane Lucas</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="n">
+        <v>168</v>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Babe veut une côte de veau à la Milanaise 🥩🇮🇹🍝 Yessss chef ! @Andy Cooks  Ingrédients (pour 2 p</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>...e détende à température ambiante. - Avec du papier cuisson ou du film alimentaire couvrir la viande. - Frapper dessus avec un rouleau à pâtisserie pour aplatir la viande au maximum. - Saler et poivrer et réserver. - Dans un récipient broyer les biscottes pour en faire de la poudre. - Ajouter du parmesan, zests de citron jaune, sel et poivre. - Paner la côte en commençant par la farine, puis les œufs et enfin la panure. - Dans une</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J80" s="8" t="inlineStr"/>
+      <c r="K80" s="8" t="inlineStr"/>
+    </row>
+    <row r="81" ht="108" customHeight="1">
+      <c r="A81" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Toscane Lucas</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="n">
+        <v>168</v>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Babe veut une côte de veau à la Milanaise 🥩🇮🇹🍝 Yessss chef ! @Andy Cooks  Ingrédients (pour 2 p</t>
+        </is>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>...e détende à température ambiante. - Avec du papier cuisson ou du film alimentaire couvrir la viande. - Frapper dessus avec un rouleau à pâtisserie pour aplatir la viande au maximum. - Saler et poivrer et réserver. - Dans un récipient broyer les biscottes pour en faire de la poudre. - Ajouter du parmesan, zests de citron jaune, sel et poivre. - Paner la côte en commençant par la farine, puis les œufs et enfin la panure. - Dans une</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J81" s="8" t="inlineStr"/>
+      <c r="K81" s="8" t="inlineStr"/>
+    </row>
+    <row r="82" ht="108" customHeight="1">
+      <c r="A82" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Toscane Lucas</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="n">
+        <v>168</v>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-09</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Babe veut des tacos 🌮🇲🇽🪅 Yessss chef ! @Andy Cooks  Musique : Mexico Cruise - DJ Zone Ingrédien</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>...s à tenir sur la viande. - Dans une cocotte colorer chaque face de la viande. - Ajouter les oignons blancs coupés en 4, les jalapeno coupé</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J82" s="8" t="inlineStr"/>
+      <c r="K82" s="8" t="inlineStr"/>
+    </row>
+    <row r="83" ht="108" customHeight="1">
+      <c r="A83" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Oh! La vie Est belle</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>2023-02-02</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Crêpes sarrasin</t>
+        </is>
+      </c>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>Le sarrasin est naturellement sans gluten et cette recette se réalise sans produits laitiers, voici donc une recette de crêpes idéales pour les personnes souffrant de troubles digestifs:
+—
+Pour environ 5/6 crêpes:
+* 500 g de farine de sarrasin
+* 1 l d’eau
+* 50 cl de lait végétal de votre choix
+* 1 œuf
+* 1 pincée de sel
+* Huile de coco
+—
+Versez la farine de sarrasin dans un saladier et former un puit au milieu.
+Ajoutez</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J83" s="8" t="inlineStr"/>
+      <c r="K83" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K73"/>
+  <autoFilter ref="A1:K83"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2 J3 J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 J46 J47 J48 J49 J50 J51 J52 J53 J54 J55 J56 J57 J58 J59 J60 J61 J62 J63 J64 J65 J66 J67 J68 J69 J70 J71 J72 J73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2 J3 J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 J46 J47 J48 J49 J50 J51 J52 J53 J54 J55 J56 J57 J58 J59 J60 J61 J62 J63 J64 J65 J66 J67 J68 J69 J70 J71 J72 J73 J74 J75 J76 J77 J78 J79 J80 J81 J82 J83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"collaboration remuneree,mention sans collaboration,auto-promotion,je ne sais pas,hors sujet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4170,6 +4650,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>